<commit_message>
docs: clarify Siemens weekly plan workflow
</commit_message>
<xml_diff>
--- a/doc/西门子杯规划/11-西门子杯综合协作资料库.xlsx
+++ b/doc/西门子杯规划/11-西门子杯综合协作资料库.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06能力映射'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07策略口径'!$A$4:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08技术口径修正'!$A$4:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09周计划'!$A$4:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09周计划'!$A$4:$K$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10三人分工'!$A$4:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11原型机测试'!$A$4:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'12现场演示顺序'!$A$4:$C$11</definedName>
@@ -156,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -193,6 +193,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -559,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -704,17 +707,6 @@
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
     </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <autoFilter ref="A4:D9"/>
   <mergeCells count="2">
@@ -731,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -743,6 +735,8 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="54" customWidth="1" min="10" max="10"/>
+    <col width="54" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -771,49 +765,59 @@
       <c r="I3" s="2" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>周次</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>开始日期</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>结束日期</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>阶段</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>交付物/任务</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>负责人</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="13" t="inlineStr">
         <is>
           <t>说明</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>工作流程</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>意义与作用</t>
         </is>
       </c>
     </row>
@@ -863,6 +867,16 @@
           <t>把每个评分项对应到 PPT/PDF 章节、证据、负责人</t>
         </is>
       </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>先读评分细则，把每个评分项拆成“材料章节、需要证据、负责人、截止时间”；再和 PPT/PDF 大纲逐项对应。交付物是一张评分对齐表。</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>让大家知道每一分靠什么材料拿，避免写了很多内容但没有覆盖评分点，也方便后续检查缺口。</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -910,6 +924,16 @@
           <t>按 2026-07-15 左右比赛倒排；继续确认正式提交、报到、抽签日期</t>
         </is>
       </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>向分赛区通知、群公告或负责人确认提交截止、报到、抽签、比赛日期；确认后写到表格和群里。交付物是明确日期记录。</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>所有任务都要按真实截止时间倒排，日期不清楚会导致后面材料和演示节奏失控。</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -957,6 +981,16 @@
           <t>Web/后端/小程序/树莓派/模拟器功能证据</t>
         </is>
       </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>按 Web、后端、小程序、树莓派、模拟器逐项列出已实现功能、关键文件、能否演示、需要截图/日志。交付物是代码能力证据表。</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>保证正式材料只写真实可验证能力，研发答辩时也能快速说出代码依据。</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1004,6 +1038,16 @@
           <t>当前原型机能否运动、云台、摄像头、传感器、星闪、供电</t>
         </is>
       </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>逐项检查底盘、云台、摄像头、传感器、星闪、供电、扬声器等是否能用；拍照或记录异常。交付物是硬件自检表。</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>决定现场能演示哪些功能，避免 PPT 写得很强但样机现场跑不出来。</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1051,6 +1095,16 @@
           <t>整理关键装配、零件、导出格式</t>
         </is>
       </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>从已入库模型中挑整机装配、关键零件、STEP/SLDASM/SLDPRT/3MF 文件，标注用途和是否需要导图。交付物是模型文件清单和截图需求表。</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>三维建模是单独得分项，也支撑制造、BOM、装配和质检说明。</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1098,6 +1152,16 @@
           <t>在 07-问题清单_请回复.md 中补充真实状态</t>
         </is>
       </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>打开问题清单，按负责人补充当前真实答案、证据位置、是否仍阻塞；无法确认的写明下一步。交付物是更新后的问题清单。</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>把不确定信息集中暴露出来，减少口径冲突，也方便你和队友异步协作。</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1145,6 +1209,16 @@
           <t>机器人本体、树莓派、下位机、传感器、后端、Web、小程序、AI</t>
         </is>
       </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>根据真实链路画出机器人本体、树莓派、下位机、传感器、后端、Web、小程序、AI、云服务的关系。交付物是一张可放 PPT/PDF 的架构图。</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>技术方案 20 分的核心材料，让评委快速理解系统怎么组成、数据怎么流动。</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1192,6 +1266,16 @@
           <t>Web 指令、Socket.IO、串口下发、电机/云台响应、安全停车</t>
         </is>
       </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>把 Web 指令到后端、树莓派、串口、下位机、电机/云台的路径写清楚，并标注停止/超时逻辑。交付物是控制流程图和文字说明。</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>证明机器人不是静态展示，而是有真实控制闭环和安全策略。</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1239,6 +1323,16 @@
           <t>供电、树莓派、传感器、下位机、电机驱动、摄像头、扬声器</t>
         </is>
       </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>整理供电、树莓派、传感器、下位机、电机驱动、摄像头、扬声器等连接关系，画成接线图。交付物是电气连接图。</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>支撑工程严谨性和制造可行性，制造工程师答辩会用到。</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1286,6 +1380,16 @@
           <t>选取关键模型文件并导出截图</t>
         </is>
       </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>选择比赛要提交的模型源文件，导出整机图、爆炸图、关键结构截图，并写清文件用途。交付物是模型提交包 v1。</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>直接对应三维建模得分，也让制造章节有图可讲。</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1333,6 +1437,16 @@
           <t>区分样机成本、可量产替代件、采购风险</t>
         </is>
       </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>列出样机主要零部件、数量、单价、供应来源、可替代件和风险。交付物是 BOM/成本草表。</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>帮助说明产品可制造、可控成本，也支撑生产管理 5 分。</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1380,6 +1494,16 @@
           <t>健康、事件、设备、机器人代理、WebRTC、AI 代理</t>
         </is>
       </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>整理健康、事件、设备、机器人代理、WebRTC、AI 等接口的用途、输入输出和调用链路。交付物是接口摘要表。</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>让研发答辩有据可查，也能支撑 PDF 技术方案章节。</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1427,6 +1551,16 @@
           <t>登录、健康、视频、遥控、事件、AI 至少 4 项稳定</t>
         </is>
       </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>固定 4 个以上最稳功能，连续走通登录、健康、视频、遥控、事件或 AI；记录失败点。交付物是可跑通的演示流程。</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>现场展示靠稳定性拿分，主演示链路越短越稳越好。</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1474,6 +1608,16 @@
           <t>明确启动顺序、环境变量、日志位置</t>
         </is>
       </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>整理树莓派启动顺序、命令、环境变量、日志位置、异常重启方式。交付物是启动脚本或启动手册。</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>比赛现场出问题时能快速恢复，降低演示失败风险。</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1521,6 +1665,16 @@
           <t>电池、线束、底盘、云台、散热、外壳固定</t>
         </is>
       </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>检查电池、线束、底盘、云台、散热、外壳固定，记录问题并处理。交付物是机械检查表和照片。</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>保证实物连续演示稳定，也能支撑样机制作和品质控制。</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1568,6 +1722,16 @@
           <t>5 分钟脚本和每次彩排失败点</t>
         </is>
       </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>写 5 分钟逐秒脚本，连续彩排并记录卡顿、故障、超时、负责人和修复状态。交付物是脚本和失败点清单。</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>把演示从“临场发挥”变成可复现流程，减少比赛当天不确定性。</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1615,6 +1779,16 @@
           <t>每项都有实际结果和证据文件名</t>
         </is>
       </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>把 T01-T10 写进官方测试表，补测试方法、预期结果、实际结果、证据编号。交付物是测试表 v1。</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>现场原型机展示按测试表执行，测试表越完整越容易拿功能实现分。</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1662,6 +1836,16 @@
           <t>健康/跌倒、视频/遥控、事件提醒测试记录</t>
         </is>
       </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>对健康/跌倒、视频/遥控、事件提醒等功能录视频、截图、保存日志，并按编号命名。交付物是证据文件夹。</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>所有技术指标必须有证据，避免被专家追问时拿不出证明。</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1709,6 +1893,16 @@
           <t>市场、竞品、访谈、试用反馈、合作意向或可脱敏证明</t>
         </is>
       </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>收集养老市场数据、政策、竞品、访谈、试用反馈或合作证明，并做脱敏。交付物是市场与证明材料包。</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>市场策略和应用证明都有分值，不能只写愿景，需要真实来源支撑。</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1756,6 +1950,16 @@
           <t>按评分项组织，不写无证据指标</t>
         </is>
       </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>按评分项拼出完整 PPT 和 PDF 第一版，插入架构图、测试结果、制造、市场和 ESG 内容。交付物是可完整讲一遍的 v1。</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>越早形成完整版本，后面才有时间改逻辑、压缩时长和补证据。</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1803,6 +2007,16 @@
           <t>5 分钟版 PPT、完整方案 PDF，统一风格、压缩体积</t>
         </is>
       </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>在 v1 基础上统一风格、删无证据指标、脱敏、压缩体积并控制 5 分钟讲述。交付物是最终 PPT/PDF。</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>这是提交包最核心材料，直接影响方案展示得分。</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1850,6 +2064,16 @@
           <t>测试结果、证据编号、源文件、导出图、说明</t>
         </is>
       </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>补齐测试结果和证据编号，整理模型源文件、截图、爆炸图和说明。交付物是最终测试表与三维模型包。</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>同时支撑原型机测评和三维建模得分，是提交包硬材料。</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1897,6 +2121,16 @@
           <t>7 月 10 日可提交包，7 月 12 日前两轮彩排</t>
         </is>
       </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>完成部署演练、身份信息检查、角色问答库和压缩包命名/结构检查。交付物是可提交压缩包 v1。</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>防止因网络、环境、身份暴露、答辩角色混乱导致扣分或演示失败。</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1944,9 +2178,19 @@
           <t>不新增功能，只做命名、格式、脱敏、环境和兜底</t>
         </is>
       </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>只检查提交、设备、网络、答辩话术和兜底路线，不再新增功能或大改材料。交付物是赛前检查确认表。</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>冻结期的目标是保护稳定性，避免最后几天越改越乱。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I28"/>
+  <autoFilter ref="A4:K28"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>

</xml_diff>